<commit_message>
fixed code to align with assignment requirements
</commit_message>
<xml_diff>
--- a/Lab3/EOP_IOP.xlsx
+++ b/Lab3/EOP_IOP.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trevormm/Desktop/ENGO531/ENGO531_code/Lab3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740EF797-31C5-0C41-9128-DEADC9033DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A03A86-290E-B042-88BF-8FF17482D0B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="2280" windowWidth="27960" windowHeight="17180" xr2:uid="{B2499F7F-9E69-A84F-9278-A077D249C086}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{B2499F7F-9E69-A84F-9278-A077D249C086}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
   <si>
     <t>Image</t>
   </si>
@@ -56,27 +57,9 @@
     <t>from</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Z</t>
-  </si>
-  <si>
     <t>Point</t>
   </si>
   <si>
-    <t>deltaX</t>
-  </si>
-  <si>
-    <t>deltaY</t>
-  </si>
-  <si>
-    <t>deltaZ</t>
-  </si>
-  <si>
     <t>Missing Coordinates</t>
   </si>
   <si>
@@ -113,9 +96,6 @@
     <t>Base mm</t>
   </si>
   <si>
-    <t>c pix</t>
-  </si>
-  <si>
     <t>H/B</t>
   </si>
   <si>
@@ -149,10 +129,34 @@
     <t>portrait</t>
   </si>
   <si>
-    <t>c_mean</t>
-  </si>
-  <si>
-    <t>new name</t>
+    <t>deltaX mm</t>
+  </si>
+  <si>
+    <t>deltaY mm</t>
+  </si>
+  <si>
+    <t>deltaZ mm</t>
+  </si>
+  <si>
+    <t>X mm</t>
+  </si>
+  <si>
+    <t>Y mm</t>
+  </si>
+  <si>
+    <t>Z mm</t>
+  </si>
+  <si>
+    <t>orientation</t>
+  </si>
+  <si>
+    <t>c (pix)</t>
+  </si>
+  <si>
+    <t>c_mean (pix)</t>
+  </si>
+  <si>
+    <t>New Image name</t>
   </si>
 </sst>
 </file>
@@ -189,7 +193,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -198,61 +202,29 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -260,19 +232,23 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="medium">
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -281,23 +257,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,367 +609,369 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48FDEF3-DC5F-DE43-882C-56E4827D7EA5}">
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" customWidth="1"/>
+    <col min="7" max="7" width="7.5" customWidth="1"/>
+    <col min="8" max="8" width="6.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1097</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4">
+        <v>-45</v>
+      </c>
+      <c r="J2" s="4">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="K1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1097</v>
-      </c>
-      <c r="C2" s="1">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1">
-        <v>-45</v>
-      </c>
-      <c r="J2" s="1">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>1143</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
         <v>-3920</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="3">
         <v>-370</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <f>B15+C3</f>
         <v>-280.78719999999998</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <f>C15+D3</f>
         <v>-4149.0254999999997</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="3">
         <f>D15+E3</f>
         <v>152.2944</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>1148</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
         <v>-3520</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
         <f t="shared" ref="F4:F9" si="0">B16+C4</f>
         <v>-137.8809</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <f t="shared" ref="G4:G9" si="1">C16+D4</f>
         <v>-3613.9113000000002</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="3">
         <f t="shared" ref="H4:H9" si="2">D16+E4</f>
         <v>1227.9179999999999</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3">
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>2036</v>
       </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
         <v>-2540</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
+      <c r="E5" s="3">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3">
         <f t="shared" si="0"/>
         <v>1311.3244999999999</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <f t="shared" si="1"/>
         <v>-3712.2094999999999</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="3">
         <f t="shared" si="2"/>
         <v>415.53829999999999</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="3">
         <v>20</v>
       </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
+      <c r="J5" s="3">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3">
         <v>105</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>2045</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
+      <c r="C6" s="3">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3">
         <v>-1525</v>
       </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
         <f t="shared" si="0"/>
         <v>2228.7159000000001</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <f t="shared" si="1"/>
         <v>-3592.4672999999998</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="3">
         <f t="shared" si="2"/>
         <v>1293.5731000000001</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="3">
         <v>30</v>
       </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
+      <c r="J6" s="3">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>2045</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
+      <c r="C7" s="3">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3">
         <v>-680</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="3">
         <v>-1040</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <f t="shared" si="0"/>
         <v>2228.7159000000001</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <f t="shared" si="1"/>
         <v>-2747.4672999999998</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="3">
         <f t="shared" si="2"/>
         <v>253.57310000000007</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="3">
         <v>60</v>
       </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
+      <c r="J7" s="3">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>1106</v>
       </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3">
         <v>-980</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
         <f t="shared" si="0"/>
         <v>-1641.0098</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <f t="shared" si="1"/>
         <v>-2594.2438000000002</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="3">
         <f t="shared" si="2"/>
         <v>1587.8896</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="3">
         <v>-45</v>
       </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
+      <c r="J8" s="3">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3">
         <f>(-10)+90</f>
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>1146</v>
       </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
+      <c r="C9" s="3">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
         <v>-2285</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
         <f t="shared" si="0"/>
         <v>-162.81829999999999</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <f t="shared" si="1"/>
         <v>-2404.7968999999998</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="3">
         <f t="shared" si="2"/>
         <v>683.2079</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="L12">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>8</v>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1097</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1143</v>
       </c>
@@ -1006,7 +985,7 @@
         <v>522.2944</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1148</v>
       </c>
@@ -1091,8 +1070,8 @@
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>13</v>
+      <c r="A26" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -1137,329 +1116,328 @@
         <v>361.2389</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F32" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F32" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H32" s="5" t="s">
+      <c r="H32" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="6">
+      <c r="A33" s="5">
         <v>2</v>
       </c>
-      <c r="B33" s="7">
+      <c r="B33" s="3">
         <v>1</v>
       </c>
-      <c r="C33" s="7">
+      <c r="C33" s="3">
         <f t="shared" ref="C33:H33" si="3">F3</f>
         <v>-280.78719999999998</v>
       </c>
-      <c r="D33" s="7">
+      <c r="D33" s="3">
         <f t="shared" si="3"/>
         <v>-4149.0254999999997</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="3">
         <f t="shared" si="3"/>
         <v>152.2944</v>
       </c>
-      <c r="F33" s="7">
+      <c r="F33" s="3">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G33" s="7">
+      <c r="G33" s="3">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="3">
         <f t="shared" si="3"/>
         <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B34" s="7">
+      <c r="A34" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" s="3">
         <v>2</v>
       </c>
-      <c r="C34" s="7">
+      <c r="C34" s="3">
         <f t="shared" ref="C34:F39" si="4">F4</f>
         <v>-137.8809</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="3">
         <f t="shared" si="4"/>
         <v>-3613.9113000000002</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="3">
         <f t="shared" si="4"/>
         <v>1227.9179999999999</v>
       </c>
-      <c r="F34" s="7">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="G34" s="7">
+      <c r="F34" s="3">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G34" s="3">
         <v>-90</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="3">
         <f t="shared" ref="H34:H39" si="5">K4</f>
         <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="6">
+      <c r="A35" s="5">
         <v>4</v>
       </c>
-      <c r="B35" s="7">
+      <c r="B35" s="3">
         <v>3</v>
       </c>
-      <c r="C35" s="7">
+      <c r="C35" s="3">
         <f t="shared" si="4"/>
         <v>1311.3244999999999</v>
       </c>
-      <c r="D35" s="7">
+      <c r="D35" s="3">
         <f t="shared" si="4"/>
         <v>-3712.2094999999999</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E35" s="3">
         <f t="shared" si="4"/>
         <v>415.53829999999999</v>
       </c>
-      <c r="F35" s="7">
+      <c r="F35" s="3">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="G35" s="7">
+      <c r="G35" s="3">
         <f>J5</f>
         <v>0</v>
       </c>
-      <c r="H35" s="8">
+      <c r="H35" s="3">
         <f t="shared" si="5"/>
         <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B36" s="7">
+      <c r="A36" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="3">
         <v>4</v>
       </c>
-      <c r="C36" s="7">
+      <c r="C36" s="3">
         <f t="shared" si="4"/>
         <v>2228.7159000000001</v>
       </c>
-      <c r="D36" s="7">
+      <c r="D36" s="3">
         <f t="shared" si="4"/>
         <v>-3592.4672999999998</v>
       </c>
-      <c r="E36" s="7">
+      <c r="E36" s="3">
         <f t="shared" si="4"/>
         <v>1293.5731000000001</v>
       </c>
-      <c r="F36" s="7">
+      <c r="F36" s="3">
         <f t="shared" si="4"/>
         <v>30</v>
       </c>
-      <c r="G36" s="7">
+      <c r="G36" s="3">
         <v>-90</v>
       </c>
-      <c r="H36" s="8">
+      <c r="H36" s="3">
         <f t="shared" si="5"/>
         <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="6">
+      <c r="A37" s="5">
         <v>6</v>
       </c>
-      <c r="B37" s="7">
+      <c r="B37" s="3">
         <v>5</v>
       </c>
-      <c r="C37" s="7">
+      <c r="C37" s="3">
         <f t="shared" si="4"/>
         <v>2228.7159000000001</v>
       </c>
-      <c r="D37" s="7">
+      <c r="D37" s="3">
         <f t="shared" si="4"/>
         <v>-2747.4672999999998</v>
       </c>
-      <c r="E37" s="7">
+      <c r="E37" s="3">
         <f t="shared" si="4"/>
         <v>253.57310000000007</v>
       </c>
-      <c r="F37" s="7">
+      <c r="F37" s="3">
         <f t="shared" si="4"/>
         <v>60</v>
       </c>
-      <c r="G37" s="7">
+      <c r="G37" s="3">
         <f>J7</f>
         <v>0</v>
       </c>
-      <c r="H37" s="8">
+      <c r="H37" s="3">
         <f t="shared" si="5"/>
         <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B38" s="7">
+      <c r="A38" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" s="3">
         <v>6</v>
       </c>
-      <c r="C38" s="7">
+      <c r="C38" s="3">
         <f t="shared" si="4"/>
         <v>-1641.0098</v>
       </c>
-      <c r="D38" s="7">
+      <c r="D38" s="3">
         <f t="shared" si="4"/>
         <v>-2594.2438000000002</v>
       </c>
-      <c r="E38" s="7">
+      <c r="E38" s="3">
         <f t="shared" si="4"/>
         <v>1587.8896</v>
       </c>
-      <c r="F38" s="7">
+      <c r="F38" s="3">
         <f t="shared" si="4"/>
         <v>-45</v>
       </c>
-      <c r="G38" s="7">
+      <c r="G38" s="3">
         <v>-90</v>
       </c>
-      <c r="H38" s="8">
+      <c r="H38" s="3">
         <f t="shared" si="5"/>
         <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="6">
+      <c r="A39" s="5">
         <v>8</v>
       </c>
-      <c r="B39" s="7">
+      <c r="B39" s="3">
         <v>7</v>
       </c>
-      <c r="C39" s="7">
+      <c r="C39" s="3">
         <f t="shared" si="4"/>
         <v>-162.81829999999999</v>
       </c>
-      <c r="D39" s="7">
+      <c r="D39" s="3">
         <f t="shared" si="4"/>
         <v>-2404.7968999999998</v>
       </c>
-      <c r="E39" s="7">
+      <c r="E39" s="3">
         <f t="shared" si="4"/>
         <v>683.2079</v>
       </c>
-      <c r="F39" s="7">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="G39" s="7">
+      <c r="F39" s="3">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G39" s="3">
         <f>J9</f>
         <v>0</v>
       </c>
-      <c r="H39" s="8">
+      <c r="H39" s="3">
         <f t="shared" si="5"/>
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B40" s="10">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B40" s="3">
         <v>8</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C40" s="3">
         <f>C39</f>
         <v>-162.81829999999999</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="3">
         <f t="shared" ref="D40:H40" si="6">D39</f>
         <v>-2404.7968999999998</v>
       </c>
-      <c r="E40" s="10">
+      <c r="E40" s="3">
         <f t="shared" si="6"/>
         <v>683.2079</v>
       </c>
-      <c r="F40" s="10">
+      <c r="F40" s="3">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G40" s="10">
+      <c r="G40" s="3">
         <v>-90</v>
       </c>
-      <c r="H40" s="11">
+      <c r="H40" s="3">
         <f t="shared" si="6"/>
         <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="A43" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B43" t="s">
-        <v>22</v>
-      </c>
-      <c r="C43" t="s">
-        <v>23</v>
-      </c>
-      <c r="D43" t="s">
-        <v>25</v>
-      </c>
-      <c r="E43" t="s">
-        <v>26</v>
-      </c>
-      <c r="F43" t="s">
-        <v>24</v>
+      <c r="F43" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44">
+      <c r="A44" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="3">
         <f>89*10</f>
         <v>890</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="3">
         <f>76*10</f>
         <v>760</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="3">
         <f>B44/C44</f>
         <v>1.1710526315789473</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="3">
         <f>SQRT((D50-D51)^2+(E50-E51)^2)</f>
         <v>3469.8802038242061</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="3">
         <f>D44*E44</f>
         <v>4063.4123439520308</v>
       </c>
@@ -1469,45 +1447,46 @@
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>21</v>
-      </c>
-      <c r="B45">
+      <c r="A45" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="3">
         <f>90.5*10</f>
         <v>905</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="3">
         <f>C44</f>
         <v>760</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="3">
         <f>B45/C45</f>
         <v>1.1907894736842106</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="3">
         <f>SQRT((D52-D53)^2+(E52-E53)^2)</f>
         <v>3489.1089215538118</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="3">
         <f>D45*E45</f>
         <v>4154.7941763239469</v>
       </c>
+      <c r="G45" s="3"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C49" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E49" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
@@ -1518,7 +1497,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D50">
         <v>2358.3397163835102</v>
@@ -1527,7 +1506,7 @@
         <v>333.515604222212</v>
       </c>
       <c r="F50" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
@@ -1538,7 +1517,7 @@
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D51">
         <v>2494.2111267843402</v>
@@ -1547,7 +1526,7 @@
         <v>3800.7346034674001</v>
       </c>
       <c r="F51" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
@@ -1558,7 +1537,7 @@
         <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D52">
         <v>1614.0526088025999</v>
@@ -1567,7 +1546,7 @@
         <v>1019.59180022396</v>
       </c>
       <c r="F52" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -1578,7 +1557,7 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D53">
         <v>1814.56193222497</v>
@@ -1587,10 +1566,455 @@
         <v>4502.9346024309298</v>
       </c>
       <c r="F53" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>35</v>
       </c>
     </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" s="3">
+        <v>1</v>
+      </c>
+      <c r="B57" s="3">
+        <v>1</v>
+      </c>
+      <c r="C57" s="3">
+        <v>2358.3397163835102</v>
+      </c>
+      <c r="D57" s="3">
+        <v>333.515604222212</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" s="3">
+        <v>2</v>
+      </c>
+      <c r="B58" s="3">
+        <v>1</v>
+      </c>
+      <c r="C58" s="3">
+        <v>2494.2111267843402</v>
+      </c>
+      <c r="D58" s="3">
+        <v>3800.7346034674001</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>1</v>
+      </c>
+      <c r="B59" s="3">
+        <v>2</v>
+      </c>
+      <c r="C59" s="3">
+        <v>1614.0526088025999</v>
+      </c>
+      <c r="D59" s="3">
+        <v>1019.59180022396</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>2</v>
+      </c>
+      <c r="B60" s="3">
+        <v>2</v>
+      </c>
+      <c r="C60" s="3">
+        <v>1814.56193222497</v>
+      </c>
+      <c r="D60" s="3">
+        <v>4502.9346024309298</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C14A4EA-DF43-7743-A8FC-CDA0F6696622}">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="6.1640625" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.1640625" customWidth="1"/>
+    <col min="5" max="5" width="6.6640625" customWidth="1"/>
+    <col min="6" max="6" width="5.5" customWidth="1"/>
+    <col min="7" max="7" width="7.5" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" customWidth="1"/>
+    <col min="9" max="9" width="6.1640625" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" customWidth="1"/>
+    <col min="11" max="11" width="5.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1097</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="4">
+        <v>-45</v>
+      </c>
+      <c r="J2" s="4">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1143</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>-3920</v>
+      </c>
+      <c r="E3" s="3">
+        <v>-370</v>
+      </c>
+      <c r="F3" s="3">
+        <f>B15+C3</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
+        <f>C15+D3</f>
+        <v>-3920</v>
+      </c>
+      <c r="H3" s="3">
+        <f>D15+E3</f>
+        <v>-370</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1148</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>-3520</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <f t="shared" ref="F4:H9" si="0">B16+C4</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <f t="shared" si="0"/>
+        <v>-3520</v>
+      </c>
+      <c r="H4" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2036</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>-2540</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="3">
+        <f t="shared" si="0"/>
+        <v>-2540</v>
+      </c>
+      <c r="H5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="3">
+        <v>20</v>
+      </c>
+      <c r="J5" s="3">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2045</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>-1525</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <f t="shared" si="0"/>
+        <v>-1525</v>
+      </c>
+      <c r="H6" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="3">
+        <v>30</v>
+      </c>
+      <c r="J6" s="3">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2045</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>-680</v>
+      </c>
+      <c r="E7" s="3">
+        <v>-1040</v>
+      </c>
+      <c r="F7" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <f t="shared" si="0"/>
+        <v>-680</v>
+      </c>
+      <c r="H7" s="3">
+        <f t="shared" si="0"/>
+        <v>-1040</v>
+      </c>
+      <c r="I7" s="3">
+        <v>60</v>
+      </c>
+      <c r="J7" s="3">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1106</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>-980</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <f t="shared" si="0"/>
+        <v>-980</v>
+      </c>
+      <c r="H8" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>-45</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3">
+        <f>(-10)+90</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3">
+        <v>1146</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>-2285</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <f t="shared" si="0"/>
+        <v>-2285</v>
+      </c>
+      <c r="H9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>